<commit_message>
Modificaciones realizadas para solventar la PreCargaInicial y ciertos problemas con texto en parentesto de estudiantes, validaciones para cedulas/ruc que no permitan numeros y error en grabacion de claves para usuarios del sistema
</commit_message>
<xml_diff>
--- a/assets/plantillas/precarga_inicial_rea.xlsx
+++ b/assets/plantillas/precarga_inicial_rea.xlsx
@@ -506,7 +506,6 @@
         </is>
       </c>
     </row>
-    <row r="2"/>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -542,7 +541,6 @@
         </is>
       </c>
     </row>
-    <row r="8"/>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
@@ -571,7 +569,6 @@
         </is>
       </c>
     </row>
-    <row r="13"/>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
@@ -607,7 +604,6 @@
         </is>
       </c>
     </row>
-    <row r="19"/>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
@@ -643,7 +639,6 @@
         </is>
       </c>
     </row>
-    <row r="25"/>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
@@ -19915,8 +19910,8 @@
     <dataValidation sqref="B2:B1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no permitido" error="Seleccione uno de los valores de la lista." type="list">
       <formula1>"CEDULA,RUC,PASAPORTE"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Valor no permitido" error="Seleccione uno de los valores de la lista." type="list">
-      <formula1>"MADRE,PADRE,ABUELO,ABUELA,TIO,TIA,REPRESENTANTE LEGAL,TUTOR/A,OTRO"</formula1>
+    <dataValidation sqref="I2:I1002" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"MADRE,PADRE,ABUELO/A,HERMANO/A,TIO/A,REPRESENTANTE LEGAL,TUTOR/A,OTRO"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>